<commit_message>
Relax validator for private templates and refresh AreaMgmt files
</commit_message>
<xml_diff>
--- a/templates/Strukturvorlage_DataDictionary_v2_empty.xlsx
+++ b/templates/Strukturvorlage_DataDictionary_v2_empty.xlsx
@@ -80,7 +80,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="30">
+  <fonts count="31">
     <font>
       <name val="Aptos Narrow"/>
       <family val="2"/>
@@ -272,6 +272,13 @@
       <b val="1"/>
       <color theme="1"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <family val="2"/>
+      <b val="1"/>
+      <color theme="1"/>
+      <sz val="12"/>
     </font>
   </fonts>
   <fills count="18">
@@ -722,7 +729,7 @@
     <xf numFmtId="0" fontId="22" fillId="10" borderId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="230">
+  <cellXfs count="234">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="49" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1439,6 +1446,18 @@
     <xf numFmtId="0" fontId="7" fillId="9" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
       <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="8">
@@ -10476,269 +10495,283 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D17"/>
+  <dimension ref="A1:D18"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
-    <col width="61.5703125" bestFit="1" customWidth="1" style="228" min="1" max="1"/>
-    <col width="96.28515625" bestFit="1" customWidth="1" style="228" min="2" max="2"/>
-    <col width="11.42578125" bestFit="1" customWidth="1" style="228" min="3" max="3"/>
+    <col width="35.83203125" bestFit="1" customWidth="1" style="228" min="1" max="1"/>
+    <col width="50.6640625" bestFit="1" customWidth="1" style="228" min="2" max="2"/>
+    <col width="24.1640625" bestFit="1" customWidth="1" style="228" min="3" max="3"/>
+    <col width="50.6640625" customWidth="1" style="228" min="4" max="4"/>
+    <col width="9.1640625" customWidth="1" style="228" min="5" max="5"/>
+    <col width="9.1640625" customWidth="1" style="228" min="6" max="6"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="201" t="inlineStr">
+    <row r="1" ht="15" customHeight="1" s="228">
+      <c r="A1" s="230" t="inlineStr">
         <is>
           <t>HE-SEM Data Dictionary — Core Metadata (mandatory authoring block)</t>
         </is>
       </c>
-      <c r="B1" s="201" t="n"/>
-      <c r="C1" s="201" t="n"/>
-      <c r="D1" s="201" t="n"/>
+      <c r="B1" s="224" t="n"/>
+      <c r="C1" s="224" t="n"/>
+      <c r="D1" s="225" t="n"/>
     </row>
     <row r="2">
-      <c r="A2" s="201" t="inlineStr">
+      <c r="A2" s="224" t="inlineStr">
         <is>
           <t>Field</t>
         </is>
       </c>
-      <c r="B2" s="201" t="inlineStr">
+      <c r="B2" s="224" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
       </c>
-      <c r="C2" s="201" t="inlineStr">
+      <c r="C2" s="224" t="inlineStr">
         <is>
           <t>Requirement</t>
         </is>
       </c>
-      <c r="D2" s="201" t="inlineStr">
+      <c r="D2" s="225" t="inlineStr">
         <is>
           <t>Notes / Maps to</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="201" t="inlineStr">
+      <c r="A3" s="231" t="inlineStr">
         <is>
           <t>── IDENTIFICATION ──</t>
         </is>
       </c>
-      <c r="B3" s="201" t="n"/>
-      <c r="C3" s="201" t="n"/>
-      <c r="D3" s="201" t="n"/>
-    </row>
-    <row r="4">
-      <c r="A4" s="201" t="inlineStr">
+      <c r="B3" s="232" t="n"/>
+      <c r="C3" s="232" t="n"/>
+      <c r="D3" s="233" t="n"/>
+    </row>
+    <row r="4" ht="25.5" customHeight="1" s="228">
+      <c r="A4" s="224" t="inlineStr">
         <is>
           <t>OrganizationCode</t>
         </is>
       </c>
-      <c r="B4" s="201" t="n"/>
-      <c r="C4" s="201" t="inlineStr">
+      <c r="B4" s="224" t="n"/>
+      <c r="C4" s="224" t="inlineStr">
         <is>
           <t>REQUIRED</t>
         </is>
       </c>
-      <c r="D4" s="201" t="inlineStr">
-        <is>
-          <t>Short org code — lowercase, max 7 chars, appears in all derived IRIs</t>
+      <c r="D4" s="225" t="inlineStr">
+        <is>
+          <t>Short org code — max 6 chars, appears in all derived IRIs</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="201" t="inlineStr">
+      <c r="A5" s="224" t="inlineStr">
         <is>
           <t>DictionaryCode</t>
         </is>
       </c>
-      <c r="B5" s="201" t="n"/>
-      <c r="C5" s="201" t="inlineStr">
+      <c r="B5" s="224" t="n"/>
+      <c r="C5" s="224" t="inlineStr">
         <is>
           <t>SYSTEM-GENERATED</t>
         </is>
       </c>
-      <c r="D5" s="201" t="inlineStr">
+      <c r="D5" s="225" t="inlineStr">
         <is>
           <t>Generated from DictionaryName (EN)</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="201" t="inlineStr">
+    <row r="6" ht="25.5" customHeight="1" s="228">
+      <c r="A6" s="224" t="inlineStr">
+        <is>
+          <t>DictionaryName (EN)</t>
+        </is>
+      </c>
+      <c r="B6" s="224" t="n"/>
+      <c r="C6" s="224" t="inlineStr">
+        <is>
+          <t>REQUIRED</t>
+        </is>
+      </c>
+      <c r="D6" s="225" t="inlineStr">
+        <is>
+          <t>Required authoring title in English — source for DictionaryCode generation</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="224" t="inlineStr">
         <is>
           <t>DictionaryName (DE)</t>
         </is>
       </c>
-      <c r="B6" s="201" t="n"/>
-      <c r="C6" s="201" t="inlineStr">
+      <c r="B7" s="224" t="n"/>
+      <c r="C7" s="223" t="inlineStr">
+        <is>
+          <t>REQUIRED (min. one local language)</t>
+        </is>
+      </c>
+      <c r="D7" s="225" t="inlineStr">
+        <is>
+          <t>Core authoring title in German — minimal DCAT anchor</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="224" t="inlineStr">
+        <is>
+          <t>DictionaryName (FR)</t>
+        </is>
+      </c>
+      <c r="B8" s="224" t="n"/>
+      <c r="D8" s="225" t="inlineStr">
+        <is>
+          <t>Core authoring title in French — minimal DCAT anchor</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="224" t="inlineStr">
+        <is>
+          <t>DictionaryName (IT)</t>
+        </is>
+      </c>
+      <c r="B9" s="224" t="n"/>
+      <c r="D9" s="225" t="inlineStr">
+        <is>
+          <t>Core authoring title in Italian — minimal DCAT anchor</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="224" t="inlineStr">
+        <is>
+          <t>DictionaryVersion</t>
+        </is>
+      </c>
+      <c r="B10" s="224" t="n"/>
+      <c r="C10" s="224" t="inlineStr">
+        <is>
+          <t>REQUIRED</t>
+        </is>
+      </c>
+      <c r="D10" s="225" t="inlineStr">
+        <is>
+          <t>Semantic versioning: MAJOR.MINOR.PATCH</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="38.25" customHeight="1" s="228">
+      <c r="A11" s="224" t="inlineStr">
+        <is>
+          <t>DictionaryUri</t>
+        </is>
+      </c>
+      <c r="B11" s="224" t="n"/>
+      <c r="C11" s="224" t="inlineStr">
+        <is>
+          <t>SYSTEM-GENERATED</t>
+        </is>
+      </c>
+      <c r="D11" s="225" t="inlineStr">
+        <is>
+          <t>Derived from OrganizationCode and DictionaryCode; canonical base pattern https://example.com/&lt;OrganizationCode&gt;/&lt;DictionaryCode&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="25.5" customHeight="1" s="228">
+      <c r="A12" s="224" t="n"/>
+      <c r="B12" s="224" t="n"/>
+      <c r="C12" s="224" t="inlineStr">
+        <is>
+          <t>Guide</t>
+        </is>
+      </c>
+      <c r="D12" s="225" t="inlineStr">
+        <is>
+          <t>Private organisations may keep only this tab and delete Dictionary_public.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="231" t="inlineStr">
+        <is>
+          <t>── GOVERNANCE ──</t>
+        </is>
+      </c>
+      <c r="B13" s="232" t="n"/>
+      <c r="C13" s="232" t="n"/>
+      <c r="D13" s="233" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="224" t="inlineStr">
+        <is>
+          <t>LifecycleStatus</t>
+        </is>
+      </c>
+      <c r="B14" s="224" t="n"/>
+      <c r="C14" s="224" t="inlineStr">
+        <is>
+          <t>REQUIRED</t>
+        </is>
+      </c>
+      <c r="D14" s="225" t="inlineStr">
+        <is>
+          <t>Governance state of Data Dictionary</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="224" t="n"/>
+      <c r="B15" s="224" t="n"/>
+      <c r="C15" s="224" t="n"/>
+      <c r="D15" s="225" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="231" t="inlineStr">
+        <is>
+          <t>LEGEND:</t>
+        </is>
+      </c>
+      <c r="B16" s="232" t="n"/>
+      <c r="C16" s="232" t="n"/>
+      <c r="D16" s="233" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="224" t="inlineStr">
+        <is>
+          <t>REQUIRED</t>
+        </is>
+      </c>
+      <c r="B17" s="224" t="inlineStr">
+        <is>
+          <t>Must be filled before validation/export</t>
+        </is>
+      </c>
+      <c r="C17" s="224" t="n"/>
+      <c r="D17" s="225" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="224" t="inlineStr">
         <is>
           <t>OPTIONAL</t>
         </is>
       </c>
-      <c r="D6" s="201" t="inlineStr">
-        <is>
-          <t>Core authoring title in German — minimal DCAT/i14y anchor</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="201" t="inlineStr">
-        <is>
-          <t>DictionaryName (FR)</t>
-        </is>
-      </c>
-      <c r="B7" s="201" t="n"/>
-      <c r="C7" s="201" t="inlineStr">
-        <is>
-          <t>OPTIONAL</t>
-        </is>
-      </c>
-      <c r="D7" s="201" t="inlineStr">
-        <is>
-          <t>Optional multilingual title support</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="201" t="inlineStr">
-        <is>
-          <t>DictionaryName (EN)</t>
-        </is>
-      </c>
-      <c r="B8" s="201" t="n"/>
-      <c r="C8" s="201" t="inlineStr">
-        <is>
-          <t>REQUIRED</t>
-        </is>
-      </c>
-      <c r="D8" s="201" t="inlineStr">
-        <is>
-          <t>Required authoring title in English — source for DictionaryCode generation</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="201" t="inlineStr">
-        <is>
-          <t>DictionaryVersion</t>
-        </is>
-      </c>
-      <c r="B9" s="201" t="n"/>
-      <c r="C9" s="201" t="inlineStr">
-        <is>
-          <t>REQUIRED</t>
-        </is>
-      </c>
-      <c r="D9" s="201" t="inlineStr">
-        <is>
-          <t>Semantic versioning: MAJOR.MINOR.PATCH</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="201" t="inlineStr">
-        <is>
-          <t>DictionaryUri</t>
-        </is>
-      </c>
-      <c r="B10" s="201" t="n"/>
-      <c r="C10" s="201" t="inlineStr">
-        <is>
-          <t>SYSTEM-GENERATED</t>
-        </is>
-      </c>
-      <c r="D10" s="201" t="inlineStr">
-        <is>
-          <t>Derived from OrganizationCode and DictionaryCode; canonical base pattern https://example.com/&lt;OrganizationCode&gt;/&lt;DictionaryCode&gt;</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="201" t="n"/>
-      <c r="B11" s="201" t="n"/>
-      <c r="C11" s="201" t="inlineStr">
-        <is>
-          <t>Guide</t>
-        </is>
-      </c>
-      <c r="D11" s="201" t="inlineStr">
-        <is>
-          <t>Private organisations may keep only this tab and delete Dictionary_public.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="201" t="inlineStr">
-        <is>
-          <t>── GOVERNANCE ──</t>
-        </is>
-      </c>
-      <c r="B12" s="201" t="n"/>
-      <c r="C12" s="201" t="n"/>
-      <c r="D12" s="201" t="n"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="201" t="inlineStr">
-        <is>
-          <t>LifecycleStatus</t>
-        </is>
-      </c>
-      <c r="B13" s="201" t="n"/>
-      <c r="C13" s="201" t="inlineStr">
-        <is>
-          <t>REQUIRED</t>
-        </is>
-      </c>
-      <c r="D13" s="201" t="inlineStr">
-        <is>
-          <t>Governance state used to derive i14y registration status</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="201" t="n"/>
-      <c r="B14" s="201" t="n"/>
-      <c r="C14" s="201" t="n"/>
-      <c r="D14" s="201" t="n"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="201" t="inlineStr">
-        <is>
-          <t>LEGEND:</t>
-        </is>
-      </c>
-      <c r="B15" s="201" t="n"/>
-      <c r="C15" s="201" t="n"/>
-      <c r="D15" s="201" t="n"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="201" t="inlineStr">
-        <is>
-          <t>REQUIRED</t>
-        </is>
-      </c>
-      <c r="B16" s="201" t="inlineStr">
-        <is>
-          <t>Must be filled before validation/export</t>
-        </is>
-      </c>
-      <c r="C16" s="201" t="n"/>
-      <c r="D16" s="201" t="n"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="201" t="inlineStr">
-        <is>
-          <t>OPTIONAL</t>
-        </is>
-      </c>
-      <c r="B17" s="201" t="inlineStr">
+      <c r="B18" s="224" t="inlineStr">
         <is>
           <t>Fill if available</t>
         </is>
       </c>
-      <c r="C17" s="201" t="n"/>
-      <c r="D17" s="201" t="n"/>
+      <c r="C18" s="224" t="n"/>
+      <c r="D18" s="225" t="n"/>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="C7:C9"/>
+  </mergeCells>
   <dataValidations count="1">
     <dataValidation sqref="B13" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid LifecycleStatus" error="Please choose a value from the LifecycleStatus list." promptTitle="LifecycleStatus" prompt="Choose an allowed LifecycleStatus value." type="list">
       <formula1>=LifecycleStatus</formula1>

</xml_diff>